<commit_message>
📊 Horarios actualizados Línea 141 - 3093
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:54:15</t>
+          <t>Última actualización: 04:24:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:54:15</t>
+          <t>04:24:36</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:59</t>
+          <t>04:32</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:54:15</t>
+          <t>04:24:36</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>02:57</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01:54:15</t>
+          <t>04:24:36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:50</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>114</v>
+        <v>26</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,23 +548,273 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>01:54:15</t>
+          <t>04:24:36</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>05:10</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>46</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>05:15</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>51</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:27</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>63</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>65</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>05:39</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>75</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>81</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>05:48</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>84</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>05:56</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>92</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:14</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>110</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:18</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>114</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06:21</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>117</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -581,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,14 +844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:54:15</t>
+          <t>Última actualización: 04:24:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -635,21 +885,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:54:15</t>
+          <t>04:24:36</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:57</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -660,23 +910,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:54:15</t>
+          <t>04:24:36</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>05:27</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:24:36</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>05:56</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>92</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -706,7 +981,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:54:15</t>
+          <t>Última actualización: 04:24:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3094
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:24:36</t>
+          <t>Última actualización: 06:17:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:32</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:50</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:10</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:15</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:27</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05:39</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05:45</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05:48</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05:56</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:14</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:18</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,23 +798,98 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>117</v>
+        <v>80</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:17:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>98</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:17:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>102</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:17:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>114</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -844,7 +919,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:24:36</t>
+          <t>Última actualización: 06:17:00</t>
         </is>
       </c>
     </row>
@@ -885,12 +960,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -899,7 +974,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -910,17 +985,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:27</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -935,12 +1010,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:24:36</t>
+          <t>06:17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:56</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -949,7 +1024,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -968,7 +1043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -981,14 +1056,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:24:36</t>
+          <t>Última actualización: 06:17:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:17:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>87</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3096
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:17:00</t>
+          <t>Última actualización: 08:46:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -890,6 +890,506 @@
         <v>114</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>10</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>25</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>31</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>31</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>40</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09:31</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>45</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>52</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>55</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>57</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>69</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>70</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>72</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>83</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>85</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>87</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>100</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>101</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>117</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -906,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:17:00</t>
+          <t>Última actualización: 08:46:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1027,6 +1527,81 @@
         <v>78</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1043,7 +1618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,14 +1631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:17:00</t>
+          <t>Última actualización: 08:46:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1114,6 +1689,131 @@
         <v>87</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>102</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:46:24</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>109</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3098
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:24</t>
+          <t>Última actualización: 11:15:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1390,6 +1390,506 @@
         <v>117</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>11:16</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>10</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>12</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>23</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>26</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>26</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>37</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>40</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>42</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>53</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>65</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>72</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>79</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>83</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>85</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>86</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>101</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>13:12</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>117</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>118</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1406,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,14 +1919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:24</t>
+          <t>Última actualización: 11:15:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1602,6 +2102,81 @@
         <v>72</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>23</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>72</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1618,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1631,14 +2206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:46:24</t>
+          <t>Última actualización: 11:15:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1816,6 +2391,56 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>102</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3099
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:15:59</t>
+          <t>Última actualización: 12:31:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 76</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1723,12 +1723,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>12:40</t>
+          <t>12:35</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>12:41</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>86</v>
+        <v>5</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>101</v>
+        <v>7</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>13:12</t>
+          <t>12:40</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>117</v>
+        <v>85</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,18 +1878,493 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>86</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>11</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>24</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>25</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>26</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>13:12</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>117</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>13:13</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>42</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>11:15:59</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D62" t="n">
+      <c r="D69" t="n">
         <v>118</v>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>43</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>53</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>54</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>61</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>62</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>69</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>76</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>79</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>97</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>105</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>115</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>116</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1906,7 +2381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1919,14 +2394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:15:59</t>
+          <t>Última actualización: 12:31:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2177,6 +2652,81 @@
         <v>72</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>26</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>53</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>116</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2193,7 +2743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2206,14 +2756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:15:59</t>
+          <t>Última actualización: 12:31:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2972,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2436,9 +2986,59 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>102</v>
+        <v>26</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>57</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>12:31:45</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>81</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3100
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:31:45</t>
+          <t>Última actualización: 13:33:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 76</t>
+          <t>Total filas: 91</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>11:15:59</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>42</v>
+        <v>118</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>76</v>
+        <v>7</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>97</v>
+        <v>17</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>105</v>
+        <v>35</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>115</v>
+        <v>35</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,23 +2348,398 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>38</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>43</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>52</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>53</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
           <t>12:31:45</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>14:27</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D81" t="n">
+      <c r="D85" t="n">
         <v>116</v>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>55</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>68</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>75</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>82</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>83</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>93</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>94</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>97</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>98</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>113</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>115</v>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2381,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2394,14 +2769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:31:45</t>
+          <t>Última actualización: 13:33:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2727,6 +3102,106 @@
         <v>116</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>55</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>75</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>83</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>115</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2743,7 +3218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2756,14 +3231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:31:45</t>
+          <t>Última actualización: 13:33:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -3041,6 +3516,81 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>55</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:33:29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3101
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:29</t>
+          <t>Última actualización: 14:37:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 91</t>
+          <t>Total filas: 103</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>11:15:59</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>42</v>
+        <v>118</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,7 +2548,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>93</v>
+        <v>20</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>113</v>
+        <v>33</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,23 +2723,323 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>34</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>15:25</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>48</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>49</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
           <t>15:28</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D96" t="n">
-        <v>115</v>
-      </c>
-      <c r="E96" t="inlineStr">
+      <c r="D99" t="n">
+        <v>51</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>64</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>71</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>77</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>79</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>87</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>90</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>97</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>106</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>109</v>
+      </c>
+      <c r="E108" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2756,7 +3056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2769,14 +3069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:29</t>
+          <t>Última actualización: 14:37:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3435,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3149,7 +3449,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3185,23 +3485,48 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>15:28</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>115</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D22" t="n">
+        <v>51</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3218,7 +3543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3231,14 +3556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:29</t>
+          <t>Última actualización: 14:37:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3897,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>14:37:18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3586,11 +3911,36 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>14:37:18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>76</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3102
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:37:18</t>
+          <t>Última actualización: 15:38:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 103</t>
+          <t>Total filas: 118</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>14:37:18</t>
+          <t>15:38:31</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>14:37:18</t>
+          <t>15:38:31</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>14:37:18</t>
+          <t>15:38:31</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>14:37:18</t>
+          <t>15:38:31</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>14:37:18</t>
+          <t>15:38:31</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>14:37:18</t>
+          <t>15:38:31</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3003,16 +3003,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>106</v>
+        <v>87</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,23 +3023,398 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>29</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>33</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
           <t>14:37:18</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>97</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>45</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>47</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
         <is>
           <t>16:26</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D108" t="n">
-        <v>109</v>
-      </c>
-      <c r="E108" t="inlineStr">
+      <c r="D113" t="n">
+        <v>48</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>60</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>62</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>63</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>63</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>75</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>78</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>90</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>104</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>114</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>118</v>
+      </c>
+      <c r="E123" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3056,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3069,14 +3444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:37:18</t>
+          <t>Última actualización: 15:38:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3527,6 +3902,56 @@
         <v>51</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>90</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>114</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3543,7 +3968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3556,14 +3981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:37:18</t>
+          <t>Última actualización: 15:38:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3939,6 +4364,81 @@
         <v>76</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>17</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>60</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>85</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3103
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E123"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:38:31</t>
+          <t>Última actualización: 16:46:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 118</t>
+          <t>Total filas: 135</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>16:46:11</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>16:46:11</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>78</v>
+        <v>9</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3328,16 +3328,16 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>16:46:11</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>104</v>
+        <v>11</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>16:46:11</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>114</v>
+        <v>22</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,23 +3398,448 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>36</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>39</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
           <t>15:38:31</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>114</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>47</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>15:38:31</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
         <is>
           <t>17:36</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C127" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D123" t="n">
+      <c r="D127" t="n">
         <v>118</v>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>51</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>52</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>64</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>67</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>73</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>80</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>82</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>84</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>94</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>96</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>97</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>110</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>111</v>
+      </c>
+      <c r="E140" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3431,7 +3856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3444,14 +3869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:38:31</t>
+          <t>Última actualización: 16:46:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3910,7 +4335,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>16:46:11</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3924,7 +4349,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3952,6 +4377,81 @@
         <v>114</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>47</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>67</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>97</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3968,7 +4468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3981,14 +4481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:38:31</t>
+          <t>Última actualización: 16:46:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4922,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>16:46:11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4436,9 +4936,34 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>16:46:11</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>104</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3104
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:46:11</t>
+          <t>Última actualización: 17:32:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 135</t>
+          <t>Total filas: 144</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3462,7 +3462,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,12 +3623,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:58</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3637,7 +3637,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3653,16 +3653,16 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>82</v>
+        <v>34</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>18:22</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>96</v>
+        <v>48</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:22</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>97</v>
+        <v>50</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>110</v>
+        <v>51</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,23 +3823,248 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>53</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>64</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
           <t>18:37</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
+      <c r="C142" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D140" t="n">
+      <c r="D142" t="n">
+        <v>65</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>81</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>83</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>93</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>96</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>105</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>110</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
         <v>111</v>
       </c>
-      <c r="E140" t="inlineStr">
+      <c r="E149" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3856,7 +4081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3869,14 +4094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:46:11</t>
+          <t>Última actualización: 17:32:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4585,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>15:38:31</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4374,7 +4599,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4410,7 +4635,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4424,7 +4649,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4435,7 +4660,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4449,9 +4674,59 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>96</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>111</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4468,7 +4743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4481,14 +4756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:46:11</t>
+          <t>Última actualización: 17:32:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4947,7 +5222,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>16:46:11</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4961,11 +5236,36 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>104</v>
+        <v>58</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3105
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:32:02</t>
+          <t>Última actualización: 18:30:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 144</t>
+          <t>Total filas: 162</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3848,12 +3848,12 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>64</v>
+        <v>5</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>81</v>
+        <v>7</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>83</v>
+        <v>19</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3978,16 +3978,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>18:56</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,16 +4028,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,23 +4048,473 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>37</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
           <t>17:32:02</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>96</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>46</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>46</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>105</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>51</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>110</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>52</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
         <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C157" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D149" t="n">
+      <c r="D157" t="n">
         <v>111</v>
       </c>
-      <c r="E149" t="inlineStr">
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>55</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>70</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>70</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>73</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>85</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>92</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>98</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>98</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>112</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>114</v>
+      </c>
+      <c r="E167" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4081,7 +4531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4094,14 +4544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:32:02</t>
+          <t>Última actualización: 18:30:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -4685,12 +5135,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4699,7 +5149,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>96</v>
+        <v>37</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4715,18 +5165,93 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>96</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>52</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>17:32:02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D31" t="n">
         <v>111</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>98</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4743,7 +5268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4756,14 +5281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:32:02</t>
+          <t>Última actualización: 18:30:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -5247,25 +5772,100 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>19:01</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>31</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>17:32:02</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>19:02</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D26" t="n">
         <v>90</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>91</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3106
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:30:53</t>
+          <t>Última actualización: 19:30:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 162</t>
+          <t>Total filas: 177</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>11:15:59</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>42</v>
+        <v>118</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>110</v>
+        <v>52</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>73</v>
+        <v>10</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>92</v>
+        <v>13</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>20:08</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>98</v>
+        <v>25</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>20:08</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>98</v>
+        <v>32</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,23 +4498,398 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>33</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>35</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
           <t>18:30:53</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>98</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>20:08</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>98</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>112</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>53</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>18:30:53</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
         <is>
           <t>20:24</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
+      <c r="C173" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D167" t="n">
+      <c r="D173" t="n">
         <v>114</v>
       </c>
-      <c r="E167" t="inlineStr">
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>55</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>66</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>72</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>75</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>20:52</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>82</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>90</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>93</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>100</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>116</v>
+      </c>
+      <c r="E182" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4531,7 +4906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4544,14 +4919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:30:53</t>
+          <t>Última actualización: 19:30:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5235,23 +5610,73 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>35</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>18:30:53</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>20:08</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D33" t="n">
         <v>98</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>72</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5268,7 +5693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5281,14 +5706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:30:53</t>
+          <t>Última actualización: 19:30:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5864,6 +6289,56 @@
         <v>91</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>32</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>19:30:04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>72</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3107
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E182"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:30:04</t>
+          <t>Última actualización: 20:30:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 177</t>
+          <t>Total filas: 186</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>11:15:59</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>118</v>
+        <v>42</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>11:15:59</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>42</v>
+        <v>118</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>17:32:02</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>52</v>
+        <v>110</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>17:32:02</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4233,11 +4233,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>110</v>
+        <v>52</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4448,7 +4448,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4458,11 +4458,11 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>32</v>
+        <v>92</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>20:30:29</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,12 +4723,12 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>20:30:29</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4753,16 +4753,16 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>20:30:29</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>20:52</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>20:30:29</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>90</v>
+        <v>22</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>20:30:29</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>93</v>
+        <v>26</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,23 +4873,248 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>32</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
           <t>19:30:04</t>
         </is>
       </c>
-      <c r="B182" t="inlineStr">
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>93</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>40</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
         <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr">
+      <c r="C185" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D182" t="n">
-        <v>116</v>
-      </c>
-      <c r="E182" t="inlineStr">
+      <c r="D185" t="n">
+        <v>56</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>64</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>70</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>76</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>21:57</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>87</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>22:04</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>94</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>101</v>
+      </c>
+      <c r="E191" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4906,7 +5131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4919,14 +5144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:30:04</t>
+          <t>Última actualización: 20:30:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5660,23 +5885,48 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>11</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>19:30:04</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D35" t="n">
         <v>72</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5693,7 +5943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5706,14 +5956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:30:04</t>
+          <t>Última actualización: 20:30:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6572,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>20:30:29</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6336,11 +6586,61 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>56</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20:30:29</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>106</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3108
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-23.xlsx
+++ b/data/horarios-141-2026-05-23.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E191"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:29</t>
+          <t>Última actualización: 22:31:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 186</t>
+          <t>Total filas: 195</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>13:33:29</t>
+          <t>12:31:45</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>12:31:45</t>
+          <t>13:33:29</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>19:30:04</t>
+          <t>18:30:53</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>18:30:53</t>
+          <t>19:30:04</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -5115,6 +5115,231 @@
         <v>101</v>
       </c>
       <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>2</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>4</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>12</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>23:11</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>40</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>23:18</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>47</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>23:36</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>65</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>68</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>23:58</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>87</v>
+      </c>
+      <c r="E200" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5131,7 +5356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5144,14 +5369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:29</t>
+          <t>Última actualización: 22:31:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -5927,6 +6152,56 @@
         <v>72</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>22:31:56</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>68</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5956,7 +6231,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:30:29</t>
+          <t>Última actualización: 22:31:56</t>
         </is>
       </c>
     </row>

</xml_diff>